<commit_message>
Remove "comment" column in TOT
</commit_message>
<xml_diff>
--- a/inst/extdata/table_of_tables.xlsx
+++ b/inst/extdata/table_of_tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u0133728\Desktop\lbstproj\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E191F329-0B68-412D-A887-BABE75C97C27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B019142-F56F-43C4-9F7C-B6B0F9ED8387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1536" yWindow="1536" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>id</t>
   </si>
@@ -40,12 +40,6 @@
   </si>
   <si>
     <t>figure</t>
-  </si>
-  <si>
-    <t>comment</t>
-  </si>
-  <si>
-    <t>(for example purpose, delete)</t>
   </si>
   <si>
     <t>fig</t>
@@ -378,15 +372,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.85546875" customWidth="1"/>
-    <col min="2" max="2" width="9.7109375" customWidth="1"/>
+    <col min="1" max="1" width="15.88671875" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" customWidth="1"/>
     <col min="4" max="4" width="65" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -399,11 +393,8 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>5</v>
-      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -411,12 +402,9 @@
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>